<commit_message>
EMPOWER study: 16-sheet formula-first workbook verified (716/716 formula cells reproduce, 13 drivers directional, 134 pasted cells inert)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012CkW3xW1KqNUtQUf3ovr6G
</commit_message>
<xml_diff>
--- a/engine/empower_study/EMPOWER_Valuation_Model_09082026_public.xlsx
+++ b/engine/empower_study/EMPOWER_Valuation_Model_09082026_public.xlsx
@@ -574,7 +574,7 @@
     <t xml:space="preserve">Beta (own-stock weekly regression vs the Dubai index)</t>
   </si>
   <si>
-    <t xml:space="preserve">Own-stock weekly regression vs DFM General Index, full listing window 25-Nov-2022..17-Jul-2026 (3.64y, inside the 2-5y band): beta 0.652, R2 0.157, n 190, SE 0.110, CI90 [0.47, 0.83] — passes the usability gate (beta_result.json) (2026-08-09)</t>
+    <t xml:space="preserve">Own-stock weekly regression vs DFMGI (DFM General Index), 2022-11-25 to 2026-07-17 (3.64 years, 190 weeks): R-squared 0.16, standard error 0.11, 90% interval [0.47, 0.83] (2026-08-09)</t>
   </si>
   <si>
     <t xml:space="preserve">Marginal cost of debt</t>
@@ -4979,7 +4979,8 @@
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="26"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5332,7 +5333,8 @@
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="0" width="15"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>